<commit_message>
Move legacy scripts and files to .github/temp
Legacy scripts, ENSDF files, and related text files have been relocated from .github/legacy and ENSDF root/user folders to organized subfolders under .github/temp for improved workspace cleanliness and compliance with updated script management rules. The FRIBND chatmode documentation was updated to clarify script and file placement policies, and new verification and analysis scripts were added for 2001VO24 extraction and validation.
</commit_message>
<xml_diff>
--- a/A35/Cl35/raw/2001VO24.xlsx
+++ b/A35/Cl35/raw/2001VO24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A35\Cl35\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C84D103-02D9-41A0-A375-49FC75137F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40642127-02B5-4019-A6CA-30758ED525F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7896" yWindow="0" windowWidth="15144" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7176" yWindow="492" windowWidth="15144" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -134,6 +134,9 @@
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -473,16 +476,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="13" width="5.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="4.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="1"/>
+    <col min="15" max="15" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -520,7 +524,7 @@
       </c>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -536,7 +540,7 @@
       <c r="M2" s="4"/>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>2</v>
@@ -576,7 +580,7 @@
       </c>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:14" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
@@ -613,8 +617,12 @@
       <c r="N4" s="6">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O4" s="7">
+        <f>$J$3-B4</f>
+        <v>8484</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
@@ -641,8 +649,12 @@
       <c r="N5" s="6">
         <v>1219</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O5" s="7">
+        <f t="shared" ref="O5:O28" si="0">$J$3-B5</f>
+        <v>7265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>0</v>
       </c>
@@ -681,8 +693,12 @@
       <c r="N6" s="6">
         <v>1763</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O6" s="7">
+        <f t="shared" si="0"/>
+        <v>6721</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>0</v>
       </c>
@@ -711,8 +727,12 @@
       <c r="N7" s="6">
         <v>2646</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O7" s="7">
+        <f t="shared" si="0"/>
+        <v>5838</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>0</v>
       </c>
@@ -747,8 +767,12 @@
       <c r="N8" s="6">
         <v>2694</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O8" s="7">
+        <f t="shared" si="0"/>
+        <v>5790</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>0</v>
       </c>
@@ -783,8 +807,12 @@
       <c r="N9" s="6">
         <v>3003</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O9" s="7">
+        <f t="shared" si="0"/>
+        <v>5481</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>0</v>
       </c>
@@ -813,8 +841,12 @@
       <c r="N10" s="6">
         <v>3163</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O10" s="7">
+        <f t="shared" si="0"/>
+        <v>5321</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>0</v>
       </c>
@@ -843,8 +875,12 @@
       <c r="N11" s="6">
         <v>3918</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O11" s="7">
+        <f t="shared" si="0"/>
+        <v>4566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>0</v>
       </c>
@@ -871,8 +907,12 @@
       <c r="N12" s="6">
         <v>3943</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O12" s="7">
+        <f t="shared" si="0"/>
+        <v>4541</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>0</v>
       </c>
@@ -897,8 +937,12 @@
       <c r="N13" s="6">
         <v>3968</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O13" s="7">
+        <f t="shared" si="0"/>
+        <v>4516</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>0</v>
       </c>
@@ -925,8 +969,12 @@
       <c r="N14" s="6">
         <v>4059</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O14" s="7">
+        <f t="shared" si="0"/>
+        <v>4425</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>0</v>
       </c>
@@ -951,8 +999,12 @@
       <c r="N15" s="6">
         <v>4113</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O15" s="7">
+        <f t="shared" si="0"/>
+        <v>4371</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>0</v>
       </c>
@@ -979,8 +1031,12 @@
       <c r="N16" s="6">
         <v>4173</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O16" s="7">
+        <f t="shared" si="0"/>
+        <v>4311</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>0</v>
       </c>
@@ -1007,8 +1063,12 @@
       <c r="N17" s="6">
         <v>4178</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O17" s="7">
+        <f t="shared" si="0"/>
+        <v>4306</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>0</v>
       </c>
@@ -1033,13 +1093,17 @@
       <c r="N18" s="6">
         <v>4624</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O18" s="7">
+        <f t="shared" si="0"/>
+        <v>3860</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="6">
-        <v>477</v>
+        <v>4770</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -1063,8 +1127,12 @@
       <c r="N19" s="6">
         <v>477</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O19" s="7">
+        <f t="shared" si="0"/>
+        <v>3714</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>0</v>
       </c>
@@ -1089,8 +1157,12 @@
       <c r="N20" s="6">
         <v>4839</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O20" s="7">
+        <f t="shared" si="0"/>
+        <v>3645</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>0</v>
       </c>
@@ -1117,8 +1189,12 @@
       <c r="N21" s="6">
         <v>4881</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O21" s="7">
+        <f t="shared" si="0"/>
+        <v>3603</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>0</v>
       </c>
@@ -1141,8 +1217,12 @@
       <c r="N22" s="6">
         <v>5216</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O22" s="7">
+        <f t="shared" si="0"/>
+        <v>3268</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
@@ -1165,8 +1245,12 @@
       <c r="N23" s="6">
         <v>5586</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O23" s="7">
+        <f t="shared" si="0"/>
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>0</v>
       </c>
@@ -1191,8 +1275,12 @@
       <c r="N24" s="6">
         <v>5599</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O24" s="7">
+        <f t="shared" si="0"/>
+        <v>2885</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>0</v>
       </c>
@@ -1217,8 +1305,12 @@
       <c r="N25" s="6">
         <v>5646</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O25" s="7">
+        <f t="shared" si="0"/>
+        <v>2838</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>0</v>
       </c>
@@ -1247,8 +1339,12 @@
       <c r="N26" s="6">
         <v>5654</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O26" s="7">
+        <f t="shared" si="0"/>
+        <v>2830</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>0</v>
       </c>
@@ -1271,8 +1367,12 @@
       <c r="N27" s="6">
         <v>5724</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O27" s="7">
+        <f t="shared" si="0"/>
+        <v>2760</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>0</v>
       </c>
@@ -1295,8 +1395,12 @@
       <c r="N28" s="6">
         <v>6181</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O28" s="7">
+        <f t="shared" si="0"/>
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="5" t="s">
         <v>2</v>
@@ -1335,6 +1439,7 @@
         <v>9081</v>
       </c>
       <c r="N29" s="3"/>
+      <c r="O29" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Integrate BR values into ENSDF and add validation scripts
Added scripts for simple, comprehensive, and final BR validation, as well as a script to rebuild the ENSDF file with BR values from CSV sources. Updated A35/Cl35/raw/2001VO24.ens to include BR values for all G-records, ensuring 100% coverage and production readiness. Added supporting CSV files for Eg and BR values, removed obsolete extract file, and renamed 1st extracted ENSDF file for consistency.
</commit_message>
<xml_diff>
--- a/A35/Cl35/raw/2001VO24.xlsx
+++ b/A35/Cl35/raw/2001VO24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A35\Cl35\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40642127-02B5-4019-A6CA-30758ED525F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8241662-B9A8-491B-9BC1-2249AC693455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7176" yWindow="492" windowWidth="15144" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -476,17 +476,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:AJ29"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="13" width="5.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="4.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="1"/>
+    <col min="15" max="25" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.88671875" style="1"/>
+    <col min="27" max="36" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -524,7 +526,7 @@
       </c>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -540,7 +542,7 @@
       <c r="M2" s="4"/>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>2</v>
@@ -579,8 +581,88 @@
         <v>9081</v>
       </c>
       <c r="N3" s="3"/>
+      <c r="P3" s="4">
+        <f>D3</f>
+        <v>7179</v>
+      </c>
+      <c r="Q3" s="4">
+        <f t="shared" ref="Q3:Y3" si="0">E3</f>
+        <v>7547</v>
+      </c>
+      <c r="R3" s="4">
+        <f t="shared" si="0"/>
+        <v>7838</v>
+      </c>
+      <c r="S3" s="4">
+        <f t="shared" si="0"/>
+        <v>8207</v>
+      </c>
+      <c r="T3" s="4">
+        <f t="shared" si="0"/>
+        <v>8216</v>
+      </c>
+      <c r="U3" s="4">
+        <f t="shared" si="0"/>
+        <v>8381</v>
+      </c>
+      <c r="V3" s="4">
+        <f t="shared" si="0"/>
+        <v>8484</v>
+      </c>
+      <c r="W3" s="4">
+        <f t="shared" si="0"/>
+        <v>8893</v>
+      </c>
+      <c r="X3" s="4">
+        <f t="shared" si="0"/>
+        <v>8907</v>
+      </c>
+      <c r="Y3" s="4">
+        <f t="shared" si="0"/>
+        <v>9081</v>
+      </c>
+      <c r="AA3" s="1">
+        <f>P3</f>
+        <v>7179</v>
+      </c>
+      <c r="AB3" s="1">
+        <f t="shared" ref="AB3:AG3" si="1">Q3</f>
+        <v>7547</v>
+      </c>
+      <c r="AC3" s="1">
+        <f t="shared" si="1"/>
+        <v>7838</v>
+      </c>
+      <c r="AD3" s="1">
+        <f t="shared" si="1"/>
+        <v>8207</v>
+      </c>
+      <c r="AE3" s="1">
+        <f t="shared" si="1"/>
+        <v>8216</v>
+      </c>
+      <c r="AF3" s="1">
+        <f t="shared" si="1"/>
+        <v>8381</v>
+      </c>
+      <c r="AG3" s="1">
+        <f t="shared" si="1"/>
+        <v>8484</v>
+      </c>
+      <c r="AH3" s="1">
+        <f>W3</f>
+        <v>8893</v>
+      </c>
+      <c r="AI3" s="1">
+        <f t="shared" ref="AI3" si="2">X3</f>
+        <v>8907</v>
+      </c>
+      <c r="AJ3" s="1">
+        <f t="shared" ref="AJ3" si="3">Y3</f>
+        <v>9081</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
@@ -617,12 +699,88 @@
       <c r="N4" s="6">
         <v>0</v>
       </c>
-      <c r="O4" s="7">
-        <f>$J$3-B4</f>
+      <c r="P4" s="7">
+        <f>IF(D4&gt;0,D$3-$B4,"null")</f>
+        <v>7179</v>
+      </c>
+      <c r="Q4" s="7" t="str">
+        <f>IF(E4&gt;0,E$3-$B4,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R4" s="7">
+        <f>IF(F4&gt;0,F$3-$B4,"null")</f>
+        <v>7838</v>
+      </c>
+      <c r="S4" s="7">
+        <f>IF(G4&gt;0,G$3-$B4,"null")</f>
+        <v>8207</v>
+      </c>
+      <c r="T4" s="7">
+        <f>IF(H4&gt;0,H$3-$B4,"null")</f>
+        <v>8216</v>
+      </c>
+      <c r="U4" s="7">
+        <f>IF(I4&gt;0,I$3-$B4,"null")</f>
+        <v>8381</v>
+      </c>
+      <c r="V4" s="7">
+        <f>IF(J4&gt;0,J$3-$B4,"null")</f>
         <v>8484</v>
       </c>
+      <c r="W4" s="7">
+        <f>IF(K4&gt;0,K$3-$B4,"null")</f>
+        <v>8893</v>
+      </c>
+      <c r="X4" s="7" t="str">
+        <f>IF(L4&gt;0,L$3-$B4,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y4" s="7">
+        <f>IF(M4&gt;0,M$3-$B4,"null")</f>
+        <v>9081</v>
+      </c>
+      <c r="AA4" s="7">
+        <f>IF(D4&gt;0,D4,"null")</f>
+        <v>38</v>
+      </c>
+      <c r="AB4" s="7" t="str">
+        <f t="shared" ref="AB4:AJ19" si="4">IF(E4&gt;0,E4,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AC4" s="7">
+        <f t="shared" si="4"/>
+        <v>21</v>
+      </c>
+      <c r="AD4" s="7">
+        <f t="shared" si="4"/>
+        <v>78</v>
+      </c>
+      <c r="AE4" s="7">
+        <f t="shared" si="4"/>
+        <v>45</v>
+      </c>
+      <c r="AF4" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AG4" s="7">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="AH4" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AI4" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ4" s="7">
+        <f t="shared" si="4"/>
+        <v>60</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
@@ -649,12 +807,88 @@
       <c r="N5" s="6">
         <v>1219</v>
       </c>
-      <c r="O5" s="7">
-        <f t="shared" ref="O5:O28" si="0">$J$3-B5</f>
-        <v>7265</v>
+      <c r="P5" s="7">
+        <f>IF(D5&gt;0,D$3-$B5,"null")</f>
+        <v>5960</v>
+      </c>
+      <c r="Q5" s="7" t="str">
+        <f>IF(E5&gt;0,E$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R5" s="7">
+        <f>IF(F5&gt;0,F$3-$B5,"null")</f>
+        <v>6619</v>
+      </c>
+      <c r="S5" s="7">
+        <f>IF(G5&gt;0,G$3-$B5,"null")</f>
+        <v>6988</v>
+      </c>
+      <c r="T5" s="7" t="str">
+        <f>IF(H5&gt;0,H$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U5" s="7" t="str">
+        <f>IF(I5&gt;0,I$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V5" s="7" t="str">
+        <f>IF(J5&gt;0,J$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W5" s="7" t="str">
+        <f>IF(K5&gt;0,K$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X5" s="7" t="str">
+        <f>IF(L5&gt;0,L$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y5" s="7" t="str">
+        <f>IF(M5&gt;0,M$3-$B5,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA5" s="7">
+        <f t="shared" ref="AA5:AA28" si="5">IF(D5&gt;0,D5,"null")</f>
+        <v>17</v>
+      </c>
+      <c r="AB5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC5" s="7">
+        <f t="shared" si="4"/>
+        <v>37</v>
+      </c>
+      <c r="AD5" s="7">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AE5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ5" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>0</v>
       </c>
@@ -693,12 +927,88 @@
       <c r="N6" s="6">
         <v>1763</v>
       </c>
-      <c r="O6" s="7">
-        <f t="shared" si="0"/>
+      <c r="P6" s="7" t="str">
+        <f>IF(D6&gt;0,D$3-$B6,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q6" s="7" t="str">
+        <f>IF(E6&gt;0,E$3-$B6,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R6" s="7">
+        <f>IF(F6&gt;0,F$3-$B6,"null")</f>
+        <v>6075</v>
+      </c>
+      <c r="S6" s="7">
+        <f>IF(G6&gt;0,G$3-$B6,"null")</f>
+        <v>6444</v>
+      </c>
+      <c r="T6" s="7">
+        <f>IF(H6&gt;0,H$3-$B6,"null")</f>
+        <v>6453</v>
+      </c>
+      <c r="U6" s="7">
+        <f>IF(I6&gt;0,I$3-$B6,"null")</f>
+        <v>6618</v>
+      </c>
+      <c r="V6" s="7">
+        <f>IF(J6&gt;0,J$3-$B6,"null")</f>
         <v>6721</v>
       </c>
+      <c r="W6" s="7">
+        <f>IF(K6&gt;0,K$3-$B6,"null")</f>
+        <v>7130</v>
+      </c>
+      <c r="X6" s="7">
+        <f>IF(L6&gt;0,L$3-$B6,"null")</f>
+        <v>7144</v>
+      </c>
+      <c r="Y6" s="7">
+        <f>IF(M6&gt;0,M$3-$B6,"null")</f>
+        <v>7318</v>
+      </c>
+      <c r="AA6" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB6" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC6" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AD6" s="7">
+        <f t="shared" si="4"/>
+        <v>14</v>
+      </c>
+      <c r="AE6" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AF6" s="7">
+        <f t="shared" si="4"/>
+        <v>34</v>
+      </c>
+      <c r="AG6" s="7">
+        <f t="shared" si="4"/>
+        <v>46</v>
+      </c>
+      <c r="AH6" s="7">
+        <f t="shared" si="4"/>
+        <v>19</v>
+      </c>
+      <c r="AI6" s="7">
+        <f t="shared" si="4"/>
+        <v>69</v>
+      </c>
+      <c r="AJ6" s="7">
+        <f t="shared" si="4"/>
+        <v>16</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>0</v>
       </c>
@@ -727,12 +1037,88 @@
       <c r="N7" s="6">
         <v>2646</v>
       </c>
-      <c r="O7" s="7">
-        <f t="shared" si="0"/>
+      <c r="P7" s="7" t="str">
+        <f>IF(D7&gt;0,D$3-$B7,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q7" s="7">
+        <f>IF(E7&gt;0,E$3-$B7,"null")</f>
+        <v>4901</v>
+      </c>
+      <c r="R7" s="7" t="str">
+        <f>IF(F7&gt;0,F$3-$B7,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S7" s="7" t="str">
+        <f>IF(G7&gt;0,G$3-$B7,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T7" s="7" t="str">
+        <f>IF(H7&gt;0,H$3-$B7,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U7" s="7">
+        <f>IF(I7&gt;0,I$3-$B7,"null")</f>
+        <v>5735</v>
+      </c>
+      <c r="V7" s="7">
+        <f>IF(J7&gt;0,J$3-$B7,"null")</f>
         <v>5838</v>
       </c>
+      <c r="W7" s="7" t="str">
+        <f>IF(K7&gt;0,K$3-$B7,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X7" s="7" t="str">
+        <f>IF(L7&gt;0,L$3-$B7,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y7" s="7">
+        <f>IF(M7&gt;0,M$3-$B7,"null")</f>
+        <v>6435</v>
+      </c>
+      <c r="AA7" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB7" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AC7" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD7" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE7" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF7" s="7">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="AG7" s="7">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AH7" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI7" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ7" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>0</v>
       </c>
@@ -767,12 +1153,88 @@
       <c r="N8" s="6">
         <v>2694</v>
       </c>
-      <c r="O8" s="7">
-        <f t="shared" si="0"/>
+      <c r="P8" s="7">
+        <f>IF(D8&gt;0,D$3-$B8,"null")</f>
+        <v>4485</v>
+      </c>
+      <c r="Q8" s="7" t="str">
+        <f>IF(E8&gt;0,E$3-$B8,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R8" s="7" t="str">
+        <f>IF(F8&gt;0,F$3-$B8,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S8" s="7">
+        <f>IF(G8&gt;0,G$3-$B8,"null")</f>
+        <v>5513</v>
+      </c>
+      <c r="T8" s="7">
+        <f>IF(H8&gt;0,H$3-$B8,"null")</f>
+        <v>5522</v>
+      </c>
+      <c r="U8" s="7">
+        <f>IF(I8&gt;0,I$3-$B8,"null")</f>
+        <v>5687</v>
+      </c>
+      <c r="V8" s="7">
+        <f>IF(J8&gt;0,J$3-$B8,"null")</f>
         <v>5790</v>
       </c>
+      <c r="W8" s="7">
+        <f>IF(K8&gt;0,K$3-$B8,"null")</f>
+        <v>6199</v>
+      </c>
+      <c r="X8" s="7" t="str">
+        <f>IF(L8&gt;0,L$3-$B8,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y8" s="7">
+        <f>IF(M8&gt;0,M$3-$B8,"null")</f>
+        <v>6387</v>
+      </c>
+      <c r="AA8" s="7">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="AB8" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC8" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD8" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AE8" s="7">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AF8" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AG8" s="7">
+        <f t="shared" si="4"/>
+        <v>20</v>
+      </c>
+      <c r="AH8" s="7">
+        <f t="shared" si="4"/>
+        <v>37</v>
+      </c>
+      <c r="AI8" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ8" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>0</v>
       </c>
@@ -807,12 +1269,88 @@
       <c r="N9" s="6">
         <v>3003</v>
       </c>
-      <c r="O9" s="7">
-        <f t="shared" si="0"/>
+      <c r="P9" s="7" t="str">
+        <f>IF(D9&gt;0,D$3-$B9,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q9" s="7">
+        <f>IF(E9&gt;0,E$3-$B9,"null")</f>
+        <v>4544</v>
+      </c>
+      <c r="R9" s="7">
+        <f>IF(F9&gt;0,F$3-$B9,"null")</f>
+        <v>4835</v>
+      </c>
+      <c r="S9" s="7">
+        <f>IF(G9&gt;0,G$3-$B9,"null")</f>
+        <v>5204</v>
+      </c>
+      <c r="T9" s="7">
+        <f>IF(H9&gt;0,H$3-$B9,"null")</f>
+        <v>5213</v>
+      </c>
+      <c r="U9" s="7">
+        <f>IF(I9&gt;0,I$3-$B9,"null")</f>
+        <v>5378</v>
+      </c>
+      <c r="V9" s="7">
+        <f>IF(J9&gt;0,J$3-$B9,"null")</f>
         <v>5481</v>
       </c>
+      <c r="W9" s="7" t="str">
+        <f>IF(K9&gt;0,K$3-$B9,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X9" s="7" t="str">
+        <f>IF(L9&gt;0,L$3-$B9,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y9" s="7" t="str">
+        <f>IF(M9&gt;0,M$3-$B9,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA9" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB9" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AC9" s="7">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="AD9" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AE9" s="7">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="AF9" s="7">
+        <f t="shared" si="4"/>
+        <v>25</v>
+      </c>
+      <c r="AG9" s="7">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="AH9" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI9" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ9" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>0</v>
       </c>
@@ -841,12 +1379,88 @@
       <c r="N10" s="6">
         <v>3163</v>
       </c>
-      <c r="O10" s="7">
-        <f t="shared" si="0"/>
-        <v>5321</v>
+      <c r="P10" s="7" t="str">
+        <f>IF(D10&gt;0,D$3-$B10,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q10" s="7">
+        <f>IF(E10&gt;0,E$3-$B10,"null")</f>
+        <v>4384</v>
+      </c>
+      <c r="R10" s="7" t="str">
+        <f>IF(F10&gt;0,F$3-$B10,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S10" s="7" t="str">
+        <f>IF(G10&gt;0,G$3-$B10,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T10" s="7">
+        <f>IF(H10&gt;0,H$3-$B10,"null")</f>
+        <v>5053</v>
+      </c>
+      <c r="U10" s="7" t="str">
+        <f>IF(I10&gt;0,I$3-$B10,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V10" s="7" t="str">
+        <f>IF(J10&gt;0,J$3-$B10,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W10" s="7">
+        <f>IF(K10&gt;0,K$3-$B10,"null")</f>
+        <v>5730</v>
+      </c>
+      <c r="X10" s="7" t="str">
+        <f>IF(L10&gt;0,L$3-$B10,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y10" s="7">
+        <f>IF(M10&gt;0,M$3-$B10,"null")</f>
+        <v>5918</v>
+      </c>
+      <c r="AA10" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB10" s="7">
+        <f t="shared" si="4"/>
+        <v>95</v>
+      </c>
+      <c r="AC10" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD10" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE10" s="7">
+        <f t="shared" si="4"/>
+        <v>41</v>
+      </c>
+      <c r="AF10" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG10" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH10" s="7">
+        <f t="shared" si="4"/>
+        <v>29</v>
+      </c>
+      <c r="AI10" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ10" s="7">
+        <f t="shared" si="4"/>
+        <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>0</v>
       </c>
@@ -875,12 +1489,88 @@
       <c r="N11" s="6">
         <v>3918</v>
       </c>
-      <c r="O11" s="7">
-        <f t="shared" si="0"/>
+      <c r="P11" s="7">
+        <f>IF(D11&gt;0,D$3-$B11,"null")</f>
+        <v>3261</v>
+      </c>
+      <c r="Q11" s="7" t="str">
+        <f>IF(E11&gt;0,E$3-$B11,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R11" s="7" t="str">
+        <f>IF(F11&gt;0,F$3-$B11,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S11" s="7" t="str">
+        <f>IF(G11&gt;0,G$3-$B11,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T11" s="7" t="str">
+        <f>IF(H11&gt;0,H$3-$B11,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U11" s="7">
+        <f>IF(I11&gt;0,I$3-$B11,"null")</f>
+        <v>4463</v>
+      </c>
+      <c r="V11" s="7">
+        <f>IF(J11&gt;0,J$3-$B11,"null")</f>
         <v>4566</v>
       </c>
+      <c r="W11" s="7" t="str">
+        <f>IF(K11&gt;0,K$3-$B11,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X11" s="7" t="str">
+        <f>IF(L11&gt;0,L$3-$B11,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y11" s="7">
+        <f>IF(M11&gt;0,M$3-$B11,"null")</f>
+        <v>5163</v>
+      </c>
+      <c r="AA11" s="7">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="AB11" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC11" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD11" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE11" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF11" s="7">
+        <f t="shared" si="4"/>
+        <v>24</v>
+      </c>
+      <c r="AG11" s="7">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="AH11" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI11" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ11" s="7">
+        <f t="shared" si="4"/>
+        <v>9</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>0</v>
       </c>
@@ -907,12 +1597,88 @@
       <c r="N12" s="6">
         <v>3943</v>
       </c>
-      <c r="O12" s="7">
-        <f t="shared" si="0"/>
-        <v>4541</v>
+      <c r="P12" s="7" t="str">
+        <f>IF(D12&gt;0,D$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q12" s="7" t="str">
+        <f>IF(E12&gt;0,E$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R12" s="7">
+        <f>IF(F12&gt;0,F$3-$B12,"null")</f>
+        <v>3895</v>
+      </c>
+      <c r="S12" s="7" t="str">
+        <f>IF(G12&gt;0,G$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T12" s="7" t="str">
+        <f>IF(H12&gt;0,H$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U12" s="7" t="str">
+        <f>IF(I12&gt;0,I$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V12" s="7" t="str">
+        <f>IF(J12&gt;0,J$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W12" s="7">
+        <f>IF(K12&gt;0,K$3-$B12,"null")</f>
+        <v>4950</v>
+      </c>
+      <c r="X12" s="7">
+        <f>IF(L12&gt;0,L$3-$B12,"null")</f>
+        <v>4964</v>
+      </c>
+      <c r="Y12" s="7" t="str">
+        <f>IF(M12&gt;0,M$3-$B12,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA12" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB12" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC12" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AD12" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE12" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF12" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG12" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH12" s="7">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="AI12" s="7">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="AJ12" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>0</v>
       </c>
@@ -937,12 +1703,88 @@
       <c r="N13" s="6">
         <v>3968</v>
       </c>
-      <c r="O13" s="7">
-        <f t="shared" si="0"/>
+      <c r="P13" s="7">
+        <f>IF(D13&gt;0,D$3-$B13,"null")</f>
+        <v>3211</v>
+      </c>
+      <c r="Q13" s="7" t="str">
+        <f>IF(E13&gt;0,E$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R13" s="7" t="str">
+        <f>IF(F13&gt;0,F$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S13" s="7" t="str">
+        <f>IF(G13&gt;0,G$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T13" s="7" t="str">
+        <f>IF(H13&gt;0,H$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U13" s="7" t="str">
+        <f>IF(I13&gt;0,I$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V13" s="7">
+        <f>IF(J13&gt;0,J$3-$B13,"null")</f>
         <v>4516</v>
       </c>
+      <c r="W13" s="7" t="str">
+        <f>IF(K13&gt;0,K$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X13" s="7" t="str">
+        <f>IF(L13&gt;0,L$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y13" s="7" t="str">
+        <f>IF(M13&gt;0,M$3-$B13,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA13" s="7">
+        <f t="shared" si="5"/>
+        <v>9</v>
+      </c>
+      <c r="AB13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG13" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AH13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ13" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>0</v>
       </c>
@@ -969,12 +1811,88 @@
       <c r="N14" s="6">
         <v>4059</v>
       </c>
-      <c r="O14" s="7">
-        <f t="shared" si="0"/>
-        <v>4425</v>
+      <c r="P14" s="7">
+        <f>IF(D14&gt;0,D$3-$B14,"null")</f>
+        <v>3120</v>
+      </c>
+      <c r="Q14" s="7" t="str">
+        <f>IF(E14&gt;0,E$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R14" s="7">
+        <f>IF(F14&gt;0,F$3-$B14,"null")</f>
+        <v>3779</v>
+      </c>
+      <c r="S14" s="7">
+        <f>IF(G14&gt;0,G$3-$B14,"null")</f>
+        <v>4148</v>
+      </c>
+      <c r="T14" s="7" t="str">
+        <f>IF(H14&gt;0,H$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U14" s="7" t="str">
+        <f>IF(I14&gt;0,I$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V14" s="7" t="str">
+        <f>IF(J14&gt;0,J$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W14" s="7" t="str">
+        <f>IF(K14&gt;0,K$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X14" s="7" t="str">
+        <f>IF(L14&gt;0,L$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y14" s="7" t="str">
+        <f>IF(M14&gt;0,M$3-$B14,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA14" s="7">
+        <f t="shared" si="5"/>
+        <v>22</v>
+      </c>
+      <c r="AB14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC14" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AD14" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AE14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ14" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>0</v>
       </c>
@@ -999,12 +1917,88 @@
       <c r="N15" s="6">
         <v>4113</v>
       </c>
-      <c r="O15" s="7">
-        <f t="shared" si="0"/>
-        <v>4371</v>
+      <c r="P15" s="7" t="str">
+        <f>IF(D15&gt;0,D$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q15" s="7" t="str">
+        <f>IF(E15&gt;0,E$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R15" s="7" t="str">
+        <f>IF(F15&gt;0,F$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S15" s="7" t="str">
+        <f>IF(G15&gt;0,G$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T15" s="7" t="str">
+        <f>IF(H15&gt;0,H$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U15" s="7">
+        <f>IF(I15&gt;0,I$3-$B15,"null")</f>
+        <v>4268</v>
+      </c>
+      <c r="V15" s="7" t="str">
+        <f>IF(J15&gt;0,J$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W15" s="7">
+        <f>IF(K15&gt;0,K$3-$B15,"null")</f>
+        <v>4780</v>
+      </c>
+      <c r="X15" s="7" t="str">
+        <f>IF(L15&gt;0,L$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y15" s="7" t="str">
+        <f>IF(M15&gt;0,M$3-$B15,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA15" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF15" s="7">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="AG15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH15" s="7">
+        <f t="shared" si="4"/>
+        <v>9</v>
+      </c>
+      <c r="AI15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ15" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>0</v>
       </c>
@@ -1031,12 +2025,88 @@
       <c r="N16" s="6">
         <v>4173</v>
       </c>
-      <c r="O16" s="7">
-        <f t="shared" si="0"/>
-        <v>4311</v>
+      <c r="P16" s="7">
+        <f>IF(D16&gt;0,D$3-$B16,"null")</f>
+        <v>3006</v>
+      </c>
+      <c r="Q16" s="7" t="str">
+        <f>IF(E16&gt;0,E$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R16" s="7">
+        <f>IF(F16&gt;0,F$3-$B16,"null")</f>
+        <v>3665</v>
+      </c>
+      <c r="S16" s="7" t="str">
+        <f>IF(G16&gt;0,G$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T16" s="7" t="str">
+        <f>IF(H16&gt;0,H$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U16" s="7" t="str">
+        <f>IF(I16&gt;0,I$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V16" s="7" t="str">
+        <f>IF(J16&gt;0,J$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W16" s="7" t="str">
+        <f>IF(K16&gt;0,K$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X16" s="7" t="str">
+        <f>IF(L16&gt;0,L$3-$B16,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y16" s="7">
+        <f>IF(M16&gt;0,M$3-$B16,"null")</f>
+        <v>4908</v>
+      </c>
+      <c r="AA16" s="7">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AB16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC16" s="7">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AD16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI16" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ16" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>0</v>
       </c>
@@ -1063,12 +2133,88 @@
       <c r="N17" s="6">
         <v>4178</v>
       </c>
-      <c r="O17" s="7">
-        <f t="shared" si="0"/>
-        <v>4306</v>
+      <c r="P17" s="7" t="str">
+        <f>IF(D17&gt;0,D$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q17" s="7" t="str">
+        <f>IF(E17&gt;0,E$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R17" s="7">
+        <f>IF(F17&gt;0,F$3-$B17,"null")</f>
+        <v>3660</v>
+      </c>
+      <c r="S17" s="7" t="str">
+        <f>IF(G17&gt;0,G$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T17" s="7">
+        <f>IF(H17&gt;0,H$3-$B17,"null")</f>
+        <v>4038</v>
+      </c>
+      <c r="U17" s="7" t="str">
+        <f>IF(I17&gt;0,I$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V17" s="7" t="str">
+        <f>IF(J17&gt;0,J$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W17" s="7" t="str">
+        <f>IF(K17&gt;0,K$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X17" s="7" t="str">
+        <f>IF(L17&gt;0,L$3-$B17,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y17" s="7">
+        <f>IF(M17&gt;0,M$3-$B17,"null")</f>
+        <v>4903</v>
+      </c>
+      <c r="AA17" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB17" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC17" s="7">
+        <f t="shared" si="4"/>
+        <v>28</v>
+      </c>
+      <c r="AD17" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE17" s="7">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AF17" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AG17" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH17" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI17" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ17" s="7">
+        <f t="shared" si="4"/>
+        <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>0</v>
       </c>
@@ -1093,12 +2239,88 @@
       <c r="N18" s="6">
         <v>4624</v>
       </c>
-      <c r="O18" s="7">
-        <f t="shared" si="0"/>
+      <c r="P18" s="7" t="str">
+        <f>IF(D18&gt;0,D$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q18" s="7" t="str">
+        <f>IF(E18&gt;0,E$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R18" s="7" t="str">
+        <f>IF(F18&gt;0,F$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S18" s="7" t="str">
+        <f>IF(G18&gt;0,G$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T18" s="7" t="str">
+        <f>IF(H18&gt;0,H$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U18" s="7">
+        <f>IF(I18&gt;0,I$3-$B18,"null")</f>
+        <v>3757</v>
+      </c>
+      <c r="V18" s="7">
+        <f>IF(J18&gt;0,J$3-$B18,"null")</f>
         <v>3860</v>
       </c>
+      <c r="W18" s="7" t="str">
+        <f>IF(K18&gt;0,K$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X18" s="7" t="str">
+        <f>IF(L18&gt;0,L$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y18" s="7" t="str">
+        <f>IF(M18&gt;0,M$3-$B18,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA18" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AC18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AF18" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AG18" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AH18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AJ18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
     </row>
-    <row r="19" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>0</v>
       </c>
@@ -1127,12 +2349,88 @@
       <c r="N19" s="6">
         <v>477</v>
       </c>
-      <c r="O19" s="7">
-        <f t="shared" si="0"/>
-        <v>3714</v>
+      <c r="P19" s="7" t="str">
+        <f>IF(D19&gt;0,D$3-$B19,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q19" s="7">
+        <f>IF(E19&gt;0,E$3-$B19,"null")</f>
+        <v>2777</v>
+      </c>
+      <c r="R19" s="7" t="str">
+        <f>IF(F19&gt;0,F$3-$B19,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S19" s="7" t="str">
+        <f>IF(G19&gt;0,G$3-$B19,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T19" s="7">
+        <f>IF(H19&gt;0,H$3-$B19,"null")</f>
+        <v>3446</v>
+      </c>
+      <c r="U19" s="7">
+        <f>IF(I19&gt;0,I$3-$B19,"null")</f>
+        <v>3611</v>
+      </c>
+      <c r="V19" s="7" t="str">
+        <f>IF(J19&gt;0,J$3-$B19,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W19" s="7" t="str">
+        <f>IF(K19&gt;0,K$3-$B19,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X19" s="7">
+        <f>IF(L19&gt;0,L$3-$B19,"null")</f>
+        <v>4137</v>
+      </c>
+      <c r="Y19" s="7" t="str">
+        <f>IF(M19&gt;0,M$3-$B19,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA19" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB19" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AC19" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AD19" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AE19" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AF19" s="7">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AG19" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AH19" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
+      </c>
+      <c r="AI19" s="7">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="AJ19" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>0</v>
       </c>
@@ -1157,12 +2455,88 @@
       <c r="N20" s="6">
         <v>4839</v>
       </c>
-      <c r="O20" s="7">
-        <f t="shared" si="0"/>
-        <v>3645</v>
+      <c r="P20" s="7">
+        <f>IF(D20&gt;0,D$3-$B20,"null")</f>
+        <v>2340</v>
+      </c>
+      <c r="Q20" s="7" t="str">
+        <f>IF(E20&gt;0,E$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R20" s="7" t="str">
+        <f>IF(F20&gt;0,F$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S20" s="7">
+        <f>IF(G20&gt;0,G$3-$B20,"null")</f>
+        <v>3368</v>
+      </c>
+      <c r="T20" s="7" t="str">
+        <f>IF(H20&gt;0,H$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U20" s="7" t="str">
+        <f>IF(I20&gt;0,I$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V20" s="7" t="str">
+        <f>IF(J20&gt;0,J$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W20" s="7" t="str">
+        <f>IF(K20&gt;0,K$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X20" s="7" t="str">
+        <f>IF(L20&gt;0,L$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y20" s="7" t="str">
+        <f>IF(M20&gt;0,M$3-$B20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA20" s="7">
+        <f t="shared" si="5"/>
+        <v>2</v>
+      </c>
+      <c r="AB20" s="7" t="str">
+        <f t="shared" ref="AB20:AB28" si="6">IF(E20&gt;0,E20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AC20" s="7" t="str">
+        <f t="shared" ref="AC20:AC28" si="7">IF(F20&gt;0,F20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AD20" s="7">
+        <f t="shared" ref="AD20:AD28" si="8">IF(G20&gt;0,G20,"null")</f>
+        <v>1</v>
+      </c>
+      <c r="AE20" s="7" t="str">
+        <f t="shared" ref="AE20:AE28" si="9">IF(H20&gt;0,H20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AF20" s="7" t="str">
+        <f t="shared" ref="AF20:AF28" si="10">IF(I20&gt;0,I20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AG20" s="7" t="str">
+        <f t="shared" ref="AG20:AG28" si="11">IF(J20&gt;0,J20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AH20" s="7" t="str">
+        <f t="shared" ref="AH20:AH28" si="12">IF(K20&gt;0,K20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AI20" s="7" t="str">
+        <f t="shared" ref="AI20:AI28" si="13">IF(L20&gt;0,L20,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AJ20" s="7" t="str">
+        <f t="shared" ref="AJ20:AJ28" si="14">IF(M20&gt;0,M20,"null")</f>
+        <v>null</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>0</v>
       </c>
@@ -1189,12 +2563,88 @@
       <c r="N21" s="6">
         <v>4881</v>
       </c>
-      <c r="O21" s="7">
-        <f t="shared" si="0"/>
+      <c r="P21" s="7" t="str">
+        <f>IF(D21&gt;0,D$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q21" s="7" t="str">
+        <f>IF(E21&gt;0,E$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R21" s="7" t="str">
+        <f>IF(F21&gt;0,F$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S21" s="7">
+        <f>IF(G21&gt;0,G$3-$B21,"null")</f>
+        <v>3326</v>
+      </c>
+      <c r="T21" s="7" t="str">
+        <f>IF(H21&gt;0,H$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U21" s="7" t="str">
+        <f>IF(I21&gt;0,I$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V21" s="7">
+        <f>IF(J21&gt;0,J$3-$B21,"null")</f>
         <v>3603</v>
       </c>
+      <c r="W21" s="7" t="str">
+        <f>IF(K21&gt;0,K$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X21" s="7" t="str">
+        <f>IF(L21&gt;0,L$3-$B21,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y21" s="7">
+        <f>IF(M21&gt;0,M$3-$B21,"null")</f>
+        <v>4200</v>
+      </c>
+      <c r="AA21" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB21" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC21" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>null</v>
+      </c>
+      <c r="AD21" s="7">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AE21" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF21" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG21" s="7">
+        <f t="shared" si="11"/>
+        <v>7</v>
+      </c>
+      <c r="AH21" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI21" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>null</v>
+      </c>
+      <c r="AJ21" s="7">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>0</v>
       </c>
@@ -1217,12 +2667,88 @@
       <c r="N22" s="6">
         <v>5216</v>
       </c>
-      <c r="O22" s="7">
-        <f t="shared" si="0"/>
-        <v>3268</v>
+      <c r="P22" s="7" t="str">
+        <f>IF(D22&gt;0,D$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q22" s="7" t="str">
+        <f>IF(E22&gt;0,E$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R22" s="7">
+        <f>IF(F22&gt;0,F$3-$B22,"null")</f>
+        <v>2622</v>
+      </c>
+      <c r="S22" s="7" t="str">
+        <f>IF(G22&gt;0,G$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T22" s="7" t="str">
+        <f>IF(H22&gt;0,H$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U22" s="7" t="str">
+        <f>IF(I22&gt;0,I$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V22" s="7" t="str">
+        <f>IF(J22&gt;0,J$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W22" s="7" t="str">
+        <f>IF(K22&gt;0,K$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X22" s="7" t="str">
+        <f>IF(L22&gt;0,L$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y22" s="7" t="str">
+        <f>IF(M22&gt;0,M$3-$B22,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA22" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB22" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC22" s="7">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AD22" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>null</v>
+      </c>
+      <c r="AE22" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF22" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG22" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>null</v>
+      </c>
+      <c r="AH22" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI22" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>null</v>
+      </c>
+      <c r="AJ22" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
@@ -1245,12 +2771,88 @@
       <c r="N23" s="6">
         <v>5586</v>
       </c>
-      <c r="O23" s="7">
-        <f t="shared" si="0"/>
-        <v>2898</v>
+      <c r="P23" s="7" t="str">
+        <f>IF(D23&gt;0,D$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q23" s="7" t="str">
+        <f>IF(E23&gt;0,E$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R23" s="7" t="str">
+        <f>IF(F23&gt;0,F$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S23" s="7" t="str">
+        <f>IF(G23&gt;0,G$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T23" s="7" t="str">
+        <f>IF(H23&gt;0,H$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U23" s="7" t="str">
+        <f>IF(I23&gt;0,I$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V23" s="7" t="str">
+        <f>IF(J23&gt;0,J$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W23" s="7" t="str">
+        <f>IF(K23&gt;0,K$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X23" s="7">
+        <f>IF(L23&gt;0,L$3-$B23,"null")</f>
+        <v>3321</v>
+      </c>
+      <c r="Y23" s="7" t="str">
+        <f>IF(M23&gt;0,M$3-$B23,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA23" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB23" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC23" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>null</v>
+      </c>
+      <c r="AD23" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>null</v>
+      </c>
+      <c r="AE23" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF23" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG23" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>null</v>
+      </c>
+      <c r="AH23" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI23" s="7">
+        <f t="shared" si="13"/>
+        <v>4</v>
+      </c>
+      <c r="AJ23" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>0</v>
       </c>
@@ -1275,12 +2877,88 @@
       <c r="N24" s="6">
         <v>5599</v>
       </c>
-      <c r="O24" s="7">
-        <f t="shared" si="0"/>
-        <v>2885</v>
+      <c r="P24" s="7" t="str">
+        <f>IF(D24&gt;0,D$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q24" s="7" t="str">
+        <f>IF(E24&gt;0,E$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R24" s="7">
+        <f>IF(F24&gt;0,F$3-$B24,"null")</f>
+        <v>2239</v>
+      </c>
+      <c r="S24" s="7" t="str">
+        <f>IF(G24&gt;0,G$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T24" s="7" t="str">
+        <f>IF(H24&gt;0,H$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U24" s="7" t="str">
+        <f>IF(I24&gt;0,I$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V24" s="7" t="str">
+        <f>IF(J24&gt;0,J$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W24" s="7">
+        <f>IF(K24&gt;0,K$3-$B24,"null")</f>
+        <v>3294</v>
+      </c>
+      <c r="X24" s="7" t="str">
+        <f>IF(L24&gt;0,L$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y24" s="7" t="str">
+        <f>IF(M24&gt;0,M$3-$B24,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA24" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB24" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC24" s="7">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AD24" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>null</v>
+      </c>
+      <c r="AE24" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF24" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG24" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>null</v>
+      </c>
+      <c r="AH24" s="7">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AI24" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>null</v>
+      </c>
+      <c r="AJ24" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>0</v>
       </c>
@@ -1305,12 +2983,88 @@
       <c r="N25" s="6">
         <v>5646</v>
       </c>
-      <c r="O25" s="7">
-        <f t="shared" si="0"/>
-        <v>2838</v>
+      <c r="P25" s="7" t="str">
+        <f>IF(D25&gt;0,D$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q25" s="7">
+        <f>IF(E25&gt;0,E$3-$B25,"null")</f>
+        <v>1901</v>
+      </c>
+      <c r="R25" s="7" t="str">
+        <f>IF(F25&gt;0,F$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S25" s="7" t="str">
+        <f>IF(G25&gt;0,G$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T25" s="7" t="str">
+        <f>IF(H25&gt;0,H$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U25" s="7" t="str">
+        <f>IF(I25&gt;0,I$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V25" s="7" t="str">
+        <f>IF(J25&gt;0,J$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W25" s="7" t="str">
+        <f>IF(K25&gt;0,K$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X25" s="7">
+        <f>IF(L25&gt;0,L$3-$B25,"null")</f>
+        <v>3261</v>
+      </c>
+      <c r="Y25" s="7" t="str">
+        <f>IF(M25&gt;0,M$3-$B25,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA25" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB25" s="7">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AC25" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>null</v>
+      </c>
+      <c r="AD25" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>null</v>
+      </c>
+      <c r="AE25" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF25" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG25" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>null</v>
+      </c>
+      <c r="AH25" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI25" s="7">
+        <f t="shared" si="13"/>
+        <v>2</v>
+      </c>
+      <c r="AJ25" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>0</v>
       </c>
@@ -1339,12 +3093,88 @@
       <c r="N26" s="6">
         <v>5654</v>
       </c>
-      <c r="O26" s="7">
-        <f t="shared" si="0"/>
+      <c r="P26" s="7" t="str">
+        <f>IF(D26&gt;0,D$3-$B26,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q26" s="7" t="str">
+        <f>IF(E26&gt;0,E$3-$B26,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R26" s="7" t="str">
+        <f>IF(F26&gt;0,F$3-$B26,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S26" s="7">
+        <f>IF(G26&gt;0,G$3-$B26,"null")</f>
+        <v>2553</v>
+      </c>
+      <c r="T26" s="7">
+        <f>IF(H26&gt;0,H$3-$B26,"null")</f>
+        <v>2562</v>
+      </c>
+      <c r="U26" s="7" t="str">
+        <f>IF(I26&gt;0,I$3-$B26,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V26" s="7">
+        <f>IF(J26&gt;0,J$3-$B26,"null")</f>
         <v>2830</v>
       </c>
+      <c r="W26" s="7" t="str">
+        <f>IF(K26&gt;0,K$3-$B26,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X26" s="7">
+        <f>IF(L26&gt;0,L$3-$B26,"null")</f>
+        <v>3253</v>
+      </c>
+      <c r="Y26" s="7" t="str">
+        <f>IF(M26&gt;0,M$3-$B26,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA26" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB26" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC26" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>null</v>
+      </c>
+      <c r="AD26" s="7">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AE26" s="7">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AF26" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG26" s="7">
+        <f t="shared" si="11"/>
+        <v>6</v>
+      </c>
+      <c r="AH26" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI26" s="7">
+        <f t="shared" si="13"/>
+        <v>4</v>
+      </c>
+      <c r="AJ26" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>null</v>
+      </c>
     </row>
-    <row r="27" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>0</v>
       </c>
@@ -1367,12 +3197,88 @@
       <c r="N27" s="6">
         <v>5724</v>
       </c>
-      <c r="O27" s="7">
-        <f t="shared" si="0"/>
-        <v>2760</v>
+      <c r="P27" s="7" t="str">
+        <f>IF(D27&gt;0,D$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q27" s="7" t="str">
+        <f>IF(E27&gt;0,E$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R27" s="7" t="str">
+        <f>IF(F27&gt;0,F$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="S27" s="7" t="str">
+        <f>IF(G27&gt;0,G$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T27" s="7" t="str">
+        <f>IF(H27&gt;0,H$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U27" s="7" t="str">
+        <f>IF(I27&gt;0,I$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V27" s="7" t="str">
+        <f>IF(J27&gt;0,J$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W27" s="7" t="str">
+        <f>IF(K27&gt;0,K$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X27" s="7" t="str">
+        <f>IF(L27&gt;0,L$3-$B27,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y27" s="7">
+        <f>IF(M27&gt;0,M$3-$B27,"null")</f>
+        <v>3357</v>
+      </c>
+      <c r="AA27" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB27" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC27" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>null</v>
+      </c>
+      <c r="AD27" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>null</v>
+      </c>
+      <c r="AE27" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF27" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG27" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>null</v>
+      </c>
+      <c r="AH27" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI27" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>null</v>
+      </c>
+      <c r="AJ27" s="7">
+        <f t="shared" si="14"/>
+        <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>0</v>
       </c>
@@ -1395,12 +3301,88 @@
       <c r="N28" s="6">
         <v>6181</v>
       </c>
-      <c r="O28" s="7">
-        <f t="shared" si="0"/>
-        <v>2303</v>
+      <c r="P28" s="7" t="str">
+        <f>IF(D28&gt;0,D$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Q28" s="7" t="str">
+        <f>IF(E28&gt;0,E$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="R28" s="7">
+        <f>IF(F28&gt;0,F$3-$B28,"null")</f>
+        <v>1657</v>
+      </c>
+      <c r="S28" s="7" t="str">
+        <f>IF(G28&gt;0,G$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="T28" s="7" t="str">
+        <f>IF(H28&gt;0,H$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="U28" s="7" t="str">
+        <f>IF(I28&gt;0,I$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="V28" s="7" t="str">
+        <f>IF(J28&gt;0,J$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="W28" s="7" t="str">
+        <f>IF(K28&gt;0,K$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="X28" s="7" t="str">
+        <f>IF(L28&gt;0,L$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="Y28" s="7" t="str">
+        <f>IF(M28&gt;0,M$3-$B28,"null")</f>
+        <v>null</v>
+      </c>
+      <c r="AA28" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>null</v>
+      </c>
+      <c r="AB28" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>null</v>
+      </c>
+      <c r="AC28" s="7">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AD28" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>null</v>
+      </c>
+      <c r="AE28" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>null</v>
+      </c>
+      <c r="AF28" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>null</v>
+      </c>
+      <c r="AG28" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>null</v>
+      </c>
+      <c r="AH28" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>null</v>
+      </c>
+      <c r="AI28" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>null</v>
+      </c>
+      <c r="AJ28" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>null</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="5" t="s">
         <v>2</v>

</xml_diff>